<commit_message>
Remove hydro as part of least cost dispatch
</commit_message>
<xml_diff>
--- a/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
+++ b/InputData/elec/ESUfRaLCD/Elec Sources Used for Rlbty and Lst Cst Dsptch.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Dropbox\NEXT Group\90. 개인 폴더\이지우\단기대응\202501 EPS 수요전망\V3\elec\ESUfRaLCD (완료)\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\South Korea\Models\eps-southkorea\InputData\elec\ESUfRaLCD\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88B322F4-03B2-48F9-87A5-E890F925F881}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1538532C-CEFB-4B91-98ED-C0CBD15A0577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4452" yWindow="852" windowWidth="20544" windowHeight="10932" activeTab="1" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{4A7A9C5C-85FC-43FE-AB1B-A2C5DC00E496}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -185,9 +185,6 @@
     <t>hydro</t>
   </si>
   <si>
-    <t>hydro dispatch</t>
-  </si>
-  <si>
     <t>hard coal w ccs es</t>
   </si>
   <si>
@@ -210,17 +207,20 @@
   </si>
   <si>
     <t>crude oil</t>
+  </si>
+  <si>
+    <t>hard coal power plants</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -228,20 +228,20 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
       <sz val="8"/>
-      <name val="맑은 고딕"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
@@ -267,13 +267,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="표준" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -289,9 +290,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 테마">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -329,7 +330,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -435,7 +436,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -577,7 +578,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -586,17 +587,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A1D3264-BEAA-43D0-A5CC-06C5D3B72BE0}">
   <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="69.59765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="69.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>0</v>
       </c>
@@ -604,7 +605,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:2">
       <c r="A6" t="s">
         <v>2</v>
       </c>
@@ -612,142 +613,142 @@
         <v>36</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:2">
       <c r="B7" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:2">
       <c r="B8" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:2">
       <c r="A10" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2">
       <c r="A11" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2">
       <c r="A12" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:2">
       <c r="A13" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:2">
       <c r="A14" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:2">
       <c r="A15" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:2">
       <c r="A16" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:1">
       <c r="A17" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:1">
       <c r="A18" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:1">
       <c r="A19" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:1">
       <c r="A20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:1">
       <c r="A21" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:1">
       <c r="A22" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:1">
       <c r="A23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:1">
       <c r="A24" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:1">
       <c r="A25" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:1">
       <c r="A26" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:1">
       <c r="A27" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:1">
       <c r="A28" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:1">
       <c r="A29" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:1">
       <c r="A30" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:1">
       <c r="A31" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:1">
       <c r="A32" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:1">
       <c r="A33" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:1">
       <c r="A35" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:1">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -763,15 +764,15 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:C81"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C82"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="33.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="33.140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -782,593 +783,604 @@
         <v>39</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A2" t="s">
+    <row r="2" spans="1:3">
+      <c r="A2" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
         <v>29</v>
-      </c>
-      <c r="B2" t="str">
-        <f>IF(A2="","",CONCATENATE(A2," es"))</f>
-        <v>natural gas combined cycle es</v>
-      </c>
-      <c r="C2" t="str">
-        <f>IF(A2="","",CONCATENATE(A2," power plants"))</f>
-        <v>natural gas combined cycle power plants</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
-        <v>49</v>
       </c>
       <c r="B3" t="str">
         <f>IF(A3="","",CONCATENATE(A3," es"))</f>
-        <v>hydro es</v>
+        <v>natural gas combined cycle es</v>
       </c>
       <c r="C3" t="str">
-        <f>IF(A3="","",CONCATENATE(A3," power plants"))</f>
-        <v>hydro power plants</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" ref="C3:C12" si="0">IF(A3="","",CONCATENATE(A3," power plants"))</f>
+        <v>natural gas combined cycle power plants</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="B4" t="str">
         <f>IF(A4="","",CONCATENATE(A4," es"))</f>
-        <v>petroleum es</v>
+        <v>hydro es</v>
       </c>
       <c r="C4" t="str">
-        <f>IF(A4="","",CONCATENATE(A4," power plants"))</f>
-        <v>petroleum power plants</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="0"/>
+        <v>hydro power plants</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B5" t="str">
         <f>IF(A5="","",CONCATENATE(A5," es"))</f>
+        <v>petroleum es</v>
+      </c>
+      <c r="C5" t="str">
+        <f t="shared" si="0"/>
+        <v>petroleum power plants</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B6" t="str">
+        <f>IF(A6="","",CONCATENATE(A6," es"))</f>
         <v>natural gas peaker es</v>
       </c>
-      <c r="C5" t="str">
-        <f>IF(A5="","",CONCATENATE(A5," power plants"))</f>
+      <c r="C6" t="str">
+        <f t="shared" si="0"/>
         <v>natural gas peaker power plants</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A6" t="s">
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>52</v>
+      </c>
+      <c r="B7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" si="0"/>
+        <v>hard coal w ccs power plants</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
         <v>53</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B8" t="s">
         <v>51</v>
       </c>
-      <c r="C6" t="str">
-        <f>IF(A6="","",CONCATENATE(A6," power plants"))</f>
-        <v>hard coal w ccs power plants</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A7" t="s">
+      <c r="C8" t="str">
+        <f t="shared" si="0"/>
+        <v>natural gas combined cycle w ccs power plants</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
         <v>54</v>
       </c>
-      <c r="B7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C7" t="str">
-        <f>IF(A7="","",CONCATENATE(A7," power plants"))</f>
-        <v>natural gas combined cycle w ccs power plants</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9" t="str">
+        <f t="shared" si="0"/>
+        <v>biomass w ccs power plants</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
         <v>55</v>
       </c>
-      <c r="B8" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" t="str">
-        <f>IF(A8="","",CONCATENATE(A8," power plants"))</f>
-        <v>biomass w ccs power plants</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>56</v>
-      </c>
-      <c r="B9" t="s">
+      <c r="B10" t="s">
         <v>26</v>
       </c>
-      <c r="C9" t="str">
-        <f>IF(A9="","",CONCATENATE(A9," power plants"))</f>
+      <c r="C10" t="str">
+        <f t="shared" si="0"/>
         <v>lignite w ccs power plants</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
         <v>33</v>
-      </c>
-      <c r="B10" t="str">
-        <f>IF(A10="","",CONCATENATE(A10," es"))</f>
-        <v>hydrogen combustion turbine es</v>
-      </c>
-      <c r="C10" t="str">
-        <f>IF(A10="","",CONCATENATE(A10," power plants"))</f>
-        <v>hydrogen combustion turbine power plants</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>34</v>
       </c>
       <c r="B11" t="str">
         <f>IF(A11="","",CONCATENATE(A11," es"))</f>
+        <v>hydrogen combustion turbine es</v>
+      </c>
+      <c r="C11" t="str">
+        <f t="shared" si="0"/>
+        <v>hydrogen combustion turbine power plants</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>34</v>
+      </c>
+      <c r="B12" t="str">
+        <f>IF(A12="","",CONCATENATE(A12," es"))</f>
         <v>hydrogen combined cycle es</v>
       </c>
-      <c r="C11" t="str">
-        <f>IF(A11="","",CONCATENATE(A11," power plants"))</f>
+      <c r="C12" t="str">
+        <f t="shared" si="0"/>
         <v>hydrogen combined cycle power plants</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B12" t="str">
-        <f t="shared" ref="B12:B22" si="0">IF(A12="","",CONCATENATE(A12," es"))</f>
-        <v/>
-      </c>
-      <c r="C12" t="str">
-        <f t="shared" ref="C12:C67" si="1">IF(A12="","",CONCATENATE(A12," power plants"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3">
       <c r="B13" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="B13:B23" si="1">IF(A13="","",CONCATENATE(A13," es"))</f>
         <v/>
       </c>
       <c r="C13" t="str">
+        <f t="shared" ref="C13:C68" si="2">IF(A13="","",CONCATENATE(A13," power plants"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="B14" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B14" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C14" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="B15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B15" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="B16" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="2:3">
+      <c r="B17" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.4">
-      <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C17" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="2:3">
+      <c r="B18" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="18" spans="2:3" x14ac:dyDescent="0.4">
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C18" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="2:3">
+      <c r="B19" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="19" spans="2:3" x14ac:dyDescent="0.4">
-      <c r="B19" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C19" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="2:3">
+      <c r="B20" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="20" spans="2:3" x14ac:dyDescent="0.4">
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="2:3">
+      <c r="B21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="21" spans="2:3" x14ac:dyDescent="0.4">
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C21" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="2:3">
+      <c r="B22" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="22" spans="2:3" x14ac:dyDescent="0.4">
-      <c r="B22" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
       <c r="C22" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="2:3">
+      <c r="B23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-    </row>
-    <row r="23" spans="2:3" x14ac:dyDescent="0.4">
       <c r="C23" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:3">
       <c r="C24" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="2:3">
       <c r="C25" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="2:3">
       <c r="C26" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="2:3">
       <c r="C27" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="2:3">
       <c r="C28" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="2:3">
       <c r="C29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="2:3">
       <c r="C30" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="2:3">
       <c r="C31" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="2:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="2:3">
       <c r="C32" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="3:3">
       <c r="C33" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="3:3">
       <c r="C34" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="3:3">
       <c r="C35" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="3:3">
       <c r="C36" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="3:3">
       <c r="C37" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="3:3">
       <c r="C38" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="3:3">
       <c r="C39" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="3:3">
       <c r="C40" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="3:3">
       <c r="C41" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="3:3">
       <c r="C42" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="3:3">
       <c r="C43" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="3:3">
       <c r="C44" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="45" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="3:3">
       <c r="C45" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="46" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="3:3">
       <c r="C46" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="47" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="3:3">
       <c r="C47" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="48" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="3:3">
       <c r="C48" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="49" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="3:3">
       <c r="C49" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="50" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="3:3">
       <c r="C50" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="51" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="3:3">
       <c r="C51" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="52" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="3:3">
       <c r="C52" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="53" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="3:3">
       <c r="C53" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="54" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="3:3">
       <c r="C54" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="55" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="3:3">
       <c r="C55" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="56" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="3:3">
       <c r="C56" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="57" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="3:3">
       <c r="C57" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="58" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="3:3">
       <c r="C58" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="59" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="3:3">
       <c r="C59" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="60" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="3:3">
       <c r="C60" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="61" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="3:3">
       <c r="C61" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="62" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="3:3">
       <c r="C62" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="63" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="3:3">
       <c r="C63" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="64" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="3:3">
       <c r="C64" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="65" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="3:3">
       <c r="C65" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="66" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="3:3">
       <c r="C66" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="67" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="3:3">
       <c r="C67" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="68" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="3:3">
       <c r="C68" t="str">
-        <f t="shared" ref="C68:C81" si="2">IF(A68="","",CONCATENATE(A68," power plants"))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="69" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="3:3">
       <c r="C69" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="70" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" ref="C69:C82" si="3">IF(A69="","",CONCATENATE(A69," power plants"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="3:3">
       <c r="C70" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="71" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="3:3">
       <c r="C71" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="72" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="3:3">
       <c r="C72" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="73" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="3:3">
       <c r="C73" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="74" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="3:3">
       <c r="C74" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="75" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="3:3">
       <c r="C75" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="76" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="3:3">
       <c r="C76" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="77" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="3:3">
       <c r="C77" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="78" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="3:3">
       <c r="C78" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="79" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="3:3">
       <c r="C79" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="80" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="3:3">
       <c r="C80" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-    </row>
-    <row r="81" spans="3:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="3:3">
       <c r="C81" t="str">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="3:3">
+      <c r="C82" t="str">
+        <f t="shared" si="3"/>
         <v/>
       </c>
     </row>
@@ -1383,15 +1395,15 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
-  <sheetFormatPr defaultColWidth="8.796875" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.4"/>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="2" width="30.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="40.296875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="31.09765625" bestFit="1" customWidth="1"/>
+    <col min="1" max="2" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="31.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3">
       <c r="A1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1402,7 +1414,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:3">
       <c r="A2" t="s">
         <v>41</v>
       </c>
@@ -1415,7 +1427,7 @@
         <v>hard coal dispatch</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3">
       <c r="A3" t="s">
         <v>42</v>
       </c>
@@ -1428,7 +1440,7 @@
         <v>natural gas steam turbine dispatch</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3">
       <c r="A4" t="s">
         <v>29</v>
       </c>
@@ -1441,9 +1453,9 @@
         <v>natural gas combined cycle dispatch</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" ref="B5" si="2">IF(A5="","",CONCATENATE(A5," es"))</f>
@@ -1454,94 +1466,95 @@
         <v>nuclear dispatch</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B6" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>47</v>
-      </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
+        <v>30</v>
+      </c>
+      <c r="B7" t="str">
+        <f>IF(A7="","",CONCATENATE(A7," es"))</f>
+        <v>petroleum es</v>
+      </c>
+      <c r="C7" t="str">
+        <f t="shared" ref="C7:C18" si="4">IF(A7="","",CONCATENATE(A7," dispatch"))</f>
+        <v>petroleum dispatch</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B8" t="str">
         <f>IF(A8="","",CONCATENATE(A8," es"))</f>
-        <v>petroleum es</v>
+        <v>natural gas peaker es</v>
       </c>
       <c r="C8" t="str">
-        <f>IF(A8="","",CONCATENATE(A8," dispatch"))</f>
-        <v>petroleum dispatch</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>natural gas peaker dispatch</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>43</v>
       </c>
       <c r="B9" t="str">
         <f>IF(A9="","",CONCATENATE(A9," es"))</f>
-        <v>natural gas peaker es</v>
+        <v>lignite es</v>
       </c>
       <c r="C9" t="str">
-        <f>IF(A9="","",CONCATENATE(A9," dispatch"))</f>
-        <v>natural gas peaker dispatch</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>lignite dispatch</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B10" t="str">
         <f>IF(A10="","",CONCATENATE(A10," es"))</f>
-        <v>lignite es</v>
+        <v>crude oil es</v>
       </c>
       <c r="C10" t="str">
-        <f>IF(A10="","",CONCATENATE(A10," dispatch"))</f>
-        <v>lignite dispatch</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>crude oil dispatch</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>44</v>
       </c>
       <c r="B11" t="str">
         <f>IF(A11="","",CONCATENATE(A11," es"))</f>
-        <v>crude oil es</v>
+        <v>municipal solid waste es</v>
       </c>
       <c r="C11" t="str">
-        <f>IF(A11="","",CONCATENATE(A11," dispatch"))</f>
-        <v>crude oil dispatch</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>municipal solid waste dispatch</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>44</v>
-      </c>
-      <c r="B12" t="str">
-        <f>IF(A12="","",CONCATENATE(A12," es"))</f>
-        <v>municipal solid waste es</v>
+        <v>52</v>
+      </c>
+      <c r="B12" t="s">
+        <v>50</v>
       </c>
       <c r="C12" t="str">
-        <f>IF(A12="","",CONCATENATE(A12," dispatch"))</f>
-        <v>municipal solid waste dispatch</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>hard coal w ccs dispatch</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
       <c r="A13" t="s">
         <v>53</v>
       </c>
@@ -1549,82 +1562,70 @@
         <v>51</v>
       </c>
       <c r="C13" t="str">
-        <f>IF(A13="","",CONCATENATE(A13," dispatch"))</f>
-        <v>hard coal w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>natural gas combined cycle w ccs dispatch</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
       <c r="A14" t="s">
         <v>54</v>
       </c>
       <c r="B14" t="s">
-        <v>52</v>
+        <v>25</v>
       </c>
       <c r="C14" t="str">
-        <f>IF(A14="","",CONCATENATE(A14," dispatch"))</f>
-        <v>natural gas combined cycle w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>biomass w ccs dispatch</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
       <c r="A15" t="s">
         <v>55</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C15" t="str">
-        <f>IF(A15="","",CONCATENATE(A15," dispatch"))</f>
-        <v>biomass w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>lignite w ccs dispatch</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>56</v>
-      </c>
-      <c r="B16" t="s">
-        <v>26</v>
+        <v>32</v>
+      </c>
+      <c r="B16" t="str">
+        <f>IF(A16="","",CONCATENATE(A16," es"))</f>
+        <v>small modular reactor es</v>
       </c>
       <c r="C16" t="str">
-        <f>IF(A16="","",CONCATENATE(A16," dispatch"))</f>
-        <v>lignite w ccs dispatch</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>small modular reactor dispatch</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B17" t="str">
         <f>IF(A17="","",CONCATENATE(A17," es"))</f>
-        <v>small modular reactor es</v>
+        <v>hydrogen combustion turbine es</v>
       </c>
       <c r="C17" t="str">
-        <f>IF(A17="","",CONCATENATE(A17," dispatch"))</f>
-        <v>small modular reactor dispatch</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
+        <f t="shared" si="4"/>
+        <v>hydrogen combustion turbine dispatch</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" t="str">
         <f>IF(A18="","",CONCATENATE(A18," es"))</f>
-        <v>hydrogen combustion turbine es</v>
+        <v>hydrogen combined cycle es</v>
       </c>
       <c r="C18" t="str">
-        <f>IF(A18="","",CONCATENATE(A18," dispatch"))</f>
-        <v>hydrogen combustion turbine dispatch</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
-        <v>34</v>
-      </c>
-      <c r="B19" t="str">
-        <f>IF(A19="","",CONCATENATE(A19," es"))</f>
-        <v>hydrogen combined cycle es</v>
-      </c>
-      <c r="C19" t="str">
-        <f>IF(A19="","",CONCATENATE(A19," dispatch"))</f>
+        <f t="shared" si="4"/>
         <v>hydrogen combined cycle dispatch</v>
       </c>
     </row>
@@ -1635,6 +1636,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E59C87379D9A4242BB3A95F198D6F941" ma:contentTypeVersion="4" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="07a235b40ffe2d9a960bde50f6511605">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="40f4d404-d193-41dc-bb72-733c1e774208" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="485fc8e6f691b86ce0aee9b7e82feca0" ns2:_="">
     <xsd:import namespace="40f4d404-d193-41dc-bb72-733c1e774208"/>
@@ -1778,29 +1794,37 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{879DA9CE-1883-47A7-8FDE-27B63C45AB8F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78751A1A-B83C-4556-9F9A-E7828ED9C408}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76B27113-2105-4A60-9A21-B2017D2C8EF0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{76B27113-2105-4A60-9A21-B2017D2C8EF0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{78751A1A-B83C-4556-9F9A-E7828ED9C408}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{879DA9CE-1883-47A7-8FDE-27B63C45AB8F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="40f4d404-d193-41dc-bb72-733c1e774208"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>